<commit_message>
data: backfill Open price for signal performance (2026-06-18 to 2026-08-27)
Refetches OHLC from yfinance for the 704 tickers whose evaluated signal
rows were missing an Open price (local raw cache had gone stale past
2026-06-17), then recomputes and persists Open for all 5,564 affected
rows and regenerates the daily CSV/Excel review files. Going forward,
Open is populated automatically at evaluation time by the pipeline.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/performance/daily/signal_list_2026-06-18.xlsx
+++ b/data/performance/daily/signal_list_2026-06-18.xlsx
@@ -559,7 +559,7 @@
         <v>156</v>
       </c>
       <c r="D5" t="n">
-        <v/>
+        <v>139.84</v>
       </c>
       <c r="E5" t="n">
         <v>155</v>
@@ -609,7 +609,7 @@
         <v>1500</v>
       </c>
       <c r="D6" t="n">
-        <v/>
+        <v>1495.1</v>
       </c>
       <c r="E6" t="n">
         <v>1510</v>
@@ -659,7 +659,7 @@
         <v>6250</v>
       </c>
       <c r="D7" t="n">
-        <v/>
+        <v>5902.52</v>
       </c>
       <c r="E7" t="n">
         <v>6275</v>
@@ -709,7 +709,7 @@
         <v>880</v>
       </c>
       <c r="D8" t="n">
-        <v/>
+        <v>854.3200000000001</v>
       </c>
       <c r="E8" t="n">
         <v>935</v>
@@ -759,7 +759,7 @@
         <v>1985</v>
       </c>
       <c r="D9" t="n">
-        <v/>
+        <v>1910</v>
       </c>
       <c r="E9" t="n">
         <v>1750</v>
@@ -809,7 +809,7 @@
         <v>8725</v>
       </c>
       <c r="D10" t="n">
-        <v/>
+        <v>8700</v>
       </c>
       <c r="E10" t="n">
         <v>8775</v>
@@ -859,7 +859,7 @@
         <v>458</v>
       </c>
       <c r="D11" t="n">
-        <v/>
+        <v>454</v>
       </c>
       <c r="E11" t="n">
         <v>448</v>
@@ -909,7 +909,7 @@
         <v>675</v>
       </c>
       <c r="D12" t="n">
-        <v/>
+        <v>610</v>
       </c>
       <c r="E12" t="n">
         <v>655</v>
@@ -959,7 +959,7 @@
         <v>1170</v>
       </c>
       <c r="D13" t="n">
-        <v/>
+        <v>1185</v>
       </c>
       <c r="E13" t="n">
         <v>1135</v>
@@ -1009,7 +1009,7 @@
         <v>570</v>
       </c>
       <c r="D14" t="n">
-        <v/>
+        <v>570</v>
       </c>
       <c r="E14" t="n">
         <v>570</v>
@@ -1163,7 +1163,7 @@
         <v>374</v>
       </c>
       <c r="D5" t="n">
-        <v/>
+        <v>343.12</v>
       </c>
       <c r="E5" t="n">
         <v>372</v>
@@ -1213,7 +1213,7 @@
         <v>880</v>
       </c>
       <c r="D6" t="n">
-        <v/>
+        <v>920</v>
       </c>
       <c r="E6" t="n">
         <v>825</v>
@@ -1263,7 +1263,7 @@
         <v>282</v>
       </c>
       <c r="D7" t="n">
-        <v/>
+        <v>288</v>
       </c>
       <c r="E7" t="n">
         <v>288</v>
@@ -1313,7 +1313,7 @@
         <v>161</v>
       </c>
       <c r="D8" t="n">
-        <v/>
+        <v>161</v>
       </c>
       <c r="E8" t="n">
         <v>159</v>
@@ -1363,7 +1363,7 @@
         <v>167</v>
       </c>
       <c r="D9" t="n">
-        <v/>
+        <v>168</v>
       </c>
       <c r="E9" t="n">
         <v>159</v>
@@ -1413,7 +1413,7 @@
         <v>6275</v>
       </c>
       <c r="D10" t="n">
-        <v/>
+        <v>6250</v>
       </c>
       <c r="E10" t="n">
         <v>6075</v>
@@ -1463,7 +1463,7 @@
         <v>3800</v>
       </c>
       <c r="D11" t="n">
-        <v/>
+        <v>3780</v>
       </c>
       <c r="E11" t="n">
         <v>3730</v>
@@ -1513,7 +1513,7 @@
         <v>3080</v>
       </c>
       <c r="D12" t="n">
-        <v/>
+        <v>3040</v>
       </c>
       <c r="E12" t="n">
         <v>2960</v>
@@ -1563,7 +1563,7 @@
         <v>1250</v>
       </c>
       <c r="D13" t="n">
-        <v/>
+        <v>1250</v>
       </c>
       <c r="E13" t="n">
         <v>1240</v>
@@ -1613,7 +1613,7 @@
         <v>135</v>
       </c>
       <c r="D14" t="n">
-        <v/>
+        <v>142</v>
       </c>
       <c r="E14" t="n">
         <v>116</v>
@@ -1663,7 +1663,7 @@
         <v>103</v>
       </c>
       <c r="D15" t="n">
-        <v/>
+        <v>102</v>
       </c>
       <c r="E15" t="n">
         <v>101</v>
@@ -1713,7 +1713,7 @@
         <v>715</v>
       </c>
       <c r="D16" t="n">
-        <v/>
+        <v>715</v>
       </c>
       <c r="E16" t="n">
         <v>690</v>
@@ -1763,7 +1763,7 @@
         <v>1600</v>
       </c>
       <c r="D17" t="n">
-        <v/>
+        <v>1451.39</v>
       </c>
       <c r="E17" t="n">
         <v>1660</v>
@@ -1813,7 +1813,7 @@
         <v>665</v>
       </c>
       <c r="D18" t="n">
-        <v/>
+        <v>650</v>
       </c>
       <c r="E18" t="n">
         <v>670</v>
@@ -1863,7 +1863,7 @@
         <v>1500</v>
       </c>
       <c r="D19" t="n">
-        <v/>
+        <v>1585</v>
       </c>
       <c r="E19" t="n">
         <v>1390</v>
@@ -1913,7 +1913,7 @@
         <v>2380</v>
       </c>
       <c r="D20" t="n">
-        <v/>
+        <v>2240.55</v>
       </c>
       <c r="E20" t="n">
         <v>2350</v>
@@ -1963,7 +1963,7 @@
         <v>362</v>
       </c>
       <c r="D21" t="n">
-        <v/>
+        <v>314.12</v>
       </c>
       <c r="E21" t="n">
         <v>370</v>
@@ -2013,7 +2013,7 @@
         <v>1670</v>
       </c>
       <c r="D22" t="n">
-        <v/>
+        <v>1513.46</v>
       </c>
       <c r="E22" t="n">
         <v>1680</v>
@@ -2063,7 +2063,7 @@
         <v>145</v>
       </c>
       <c r="D23" t="n">
-        <v/>
+        <v>145</v>
       </c>
       <c r="E23" t="n">
         <v>124</v>
@@ -2113,7 +2113,7 @@
         <v>156</v>
       </c>
       <c r="D24" t="n">
-        <v/>
+        <v>139.84</v>
       </c>
       <c r="E24" t="n">
         <v>155</v>
@@ -2163,7 +2163,7 @@
         <v>665</v>
       </c>
       <c r="D25" t="n">
-        <v/>
+        <v>618.39</v>
       </c>
       <c r="E25" t="n">
         <v>650</v>
@@ -2213,7 +2213,7 @@
         <v>1190</v>
       </c>
       <c r="D26" t="n">
-        <v/>
+        <v>1190</v>
       </c>
       <c r="E26" t="n">
         <v>1180</v>
@@ -2263,7 +2263,7 @@
         <v>69</v>
       </c>
       <c r="D27" t="n">
-        <v/>
+        <v>75</v>
       </c>
       <c r="E27" t="n">
         <v>75</v>
@@ -2313,7 +2313,7 @@
         <v>670</v>
       </c>
       <c r="D28" t="n">
-        <v/>
+        <v>655</v>
       </c>
       <c r="E28" t="n">
         <v>650</v>
@@ -2363,7 +2363,7 @@
         <v>6750</v>
       </c>
       <c r="D29" t="n">
-        <v/>
+        <v>6514.2</v>
       </c>
       <c r="E29" t="n">
         <v>6800</v>
@@ -2413,7 +2413,7 @@
         <v>1450</v>
       </c>
       <c r="D30" t="n">
-        <v/>
+        <v>1423.54</v>
       </c>
       <c r="E30" t="n">
         <v>1370</v>
@@ -2463,7 +2463,7 @@
         <v>3500</v>
       </c>
       <c r="D31" t="n">
-        <v/>
+        <v>3410</v>
       </c>
       <c r="E31" t="n">
         <v>2980</v>
@@ -2513,7 +2513,7 @@
         <v>186</v>
       </c>
       <c r="D32" t="n">
-        <v/>
+        <v>187</v>
       </c>
       <c r="E32" t="n">
         <v>181</v>
@@ -2563,7 +2563,7 @@
         <v>800</v>
       </c>
       <c r="D33" t="n">
-        <v/>
+        <v>795</v>
       </c>
       <c r="E33" t="n">
         <v>790</v>
@@ -2613,7 +2613,7 @@
         <v>189</v>
       </c>
       <c r="D34" t="n">
-        <v/>
+        <v>192</v>
       </c>
       <c r="E34" t="n">
         <v>191</v>
@@ -2663,7 +2663,7 @@
         <v>2600</v>
       </c>
       <c r="D35" t="n">
-        <v/>
+        <v>2600</v>
       </c>
       <c r="E35" t="n">
         <v>2640</v>
@@ -2713,7 +2713,7 @@
         <v>114</v>
       </c>
       <c r="D36" t="n">
-        <v/>
+        <v>116</v>
       </c>
       <c r="E36" t="n">
         <v>109</v>
@@ -2763,7 +2763,7 @@
         <v>2150</v>
       </c>
       <c r="D37" t="n">
-        <v/>
+        <v>2140</v>
       </c>
       <c r="E37" t="n">
         <v>2130</v>
@@ -2813,7 +2813,7 @@
         <v>6250</v>
       </c>
       <c r="D38" t="n">
-        <v/>
+        <v>5902.52</v>
       </c>
       <c r="E38" t="n">
         <v>6275</v>
@@ -2863,7 +2863,7 @@
         <v>110</v>
       </c>
       <c r="D39" t="n">
-        <v/>
+        <v>112</v>
       </c>
       <c r="E39" t="n">
         <v>106</v>
@@ -2913,7 +2913,7 @@
         <v>1750</v>
       </c>
       <c r="D40" t="n">
-        <v/>
+        <v>1523.44</v>
       </c>
       <c r="E40" t="n">
         <v>1745</v>
@@ -2963,7 +2963,7 @@
         <v>132</v>
       </c>
       <c r="D41" t="n">
-        <v/>
+        <v>129</v>
       </c>
       <c r="E41" t="n">
         <v>130</v>
@@ -3013,7 +3013,7 @@
         <v>3790</v>
       </c>
       <c r="D42" t="n">
-        <v/>
+        <v>744.42</v>
       </c>
       <c r="E42" t="n">
         <v>3870</v>
@@ -3063,7 +3063,7 @@
         <v>73</v>
       </c>
       <c r="D43" t="n">
-        <v/>
+        <v>72</v>
       </c>
       <c r="E43" t="n">
         <v>70</v>
@@ -3113,7 +3113,7 @@
         <v>310</v>
       </c>
       <c r="D44" t="n">
-        <v/>
+        <v>304.76</v>
       </c>
       <c r="E44" t="n">
         <v>304</v>
@@ -3163,7 +3163,7 @@
         <v>1515</v>
       </c>
       <c r="D45" t="n">
-        <v/>
+        <v>1515</v>
       </c>
       <c r="E45" t="n">
         <v>1520</v>
@@ -3213,7 +3213,7 @@
         <v>3540</v>
       </c>
       <c r="D46" t="n">
-        <v/>
+        <v>3465.61</v>
       </c>
       <c r="E46" t="n">
         <v>3630</v>
@@ -3263,7 +3263,7 @@
         <v>650</v>
       </c>
       <c r="D47" t="n">
-        <v/>
+        <v>660</v>
       </c>
       <c r="E47" t="n">
         <v>650</v>
@@ -3313,7 +3313,7 @@
         <v>570</v>
       </c>
       <c r="D48" t="n">
-        <v/>
+        <v>560</v>
       </c>
       <c r="E48" t="n">
         <v>590</v>
@@ -3363,7 +3363,7 @@
         <v>2960</v>
       </c>
       <c r="D49" t="n">
-        <v/>
+        <v>2800</v>
       </c>
       <c r="E49" t="n">
         <v>2780</v>
@@ -3413,7 +3413,7 @@
         <v>121</v>
       </c>
       <c r="D50" t="n">
-        <v/>
+        <v>122</v>
       </c>
       <c r="E50" t="n">
         <v>118</v>
@@ -3463,7 +3463,7 @@
         <v>1085</v>
       </c>
       <c r="D51" t="n">
-        <v/>
+        <v>1085</v>
       </c>
       <c r="E51" t="n">
         <v>1080</v>
@@ -3513,7 +3513,7 @@
         <v>392</v>
       </c>
       <c r="D52" t="n">
-        <v/>
+        <v>394</v>
       </c>
       <c r="E52" t="n">
         <v>398</v>
@@ -3563,7 +3563,7 @@
         <v>545</v>
       </c>
       <c r="D53" t="n">
-        <v/>
+        <v>544.09</v>
       </c>
       <c r="E53" t="n">
         <v>540</v>
@@ -3613,7 +3613,7 @@
         <v>168</v>
       </c>
       <c r="D54" t="n">
-        <v/>
+        <v>168</v>
       </c>
       <c r="E54" t="n">
         <v>166</v>
@@ -3663,7 +3663,7 @@
         <v>1650</v>
       </c>
       <c r="D55" t="n">
-        <v/>
+        <v>1645</v>
       </c>
       <c r="E55" t="n">
         <v>1665</v>
@@ -3713,7 +3713,7 @@
         <v>1335</v>
       </c>
       <c r="D56" t="n">
-        <v/>
+        <v>1335</v>
       </c>
       <c r="E56" t="n">
         <v>1335</v>
@@ -3763,7 +3763,7 @@
         <v>880</v>
       </c>
       <c r="D57" t="n">
-        <v/>
+        <v>854.3200000000001</v>
       </c>
       <c r="E57" t="n">
         <v>935</v>
@@ -3813,7 +3813,7 @@
         <v>92</v>
       </c>
       <c r="D58" t="n">
-        <v/>
+        <v>92</v>
       </c>
       <c r="E58" t="n">
         <v>88</v>
@@ -3863,7 +3863,7 @@
         <v>6825</v>
       </c>
       <c r="D59" t="n">
-        <v/>
+        <v>6800</v>
       </c>
       <c r="E59" t="n">
         <v>6500</v>
@@ -3913,7 +3913,7 @@
         <v>187</v>
       </c>
       <c r="D60" t="n">
-        <v/>
+        <v>189</v>
       </c>
       <c r="E60" t="n">
         <v>188</v>
@@ -3963,7 +3963,7 @@
         <v>1985</v>
       </c>
       <c r="D61" t="n">
-        <v/>
+        <v>1910</v>
       </c>
       <c r="E61" t="n">
         <v>1750</v>
@@ -4013,7 +4013,7 @@
         <v>1005</v>
       </c>
       <c r="D62" t="n">
-        <v/>
+        <v>1010</v>
       </c>
       <c r="E62" t="n">
         <v>1015</v>
@@ -4063,7 +4063,7 @@
         <v>420</v>
       </c>
       <c r="D63" t="n">
-        <v/>
+        <v>420</v>
       </c>
       <c r="E63" t="n">
         <v>402</v>
@@ -4113,7 +4113,7 @@
         <v>1235</v>
       </c>
       <c r="D64" t="n">
-        <v/>
+        <v>1149.35</v>
       </c>
       <c r="E64" t="n">
         <v>1235</v>
@@ -4163,7 +4163,7 @@
         <v>177</v>
       </c>
       <c r="D65" t="n">
-        <v/>
+        <v>177</v>
       </c>
       <c r="E65" t="n">
         <v>177</v>
@@ -4213,7 +4213,7 @@
         <v>80</v>
       </c>
       <c r="D66" t="n">
-        <v/>
+        <v>78</v>
       </c>
       <c r="E66" t="n">
         <v>92</v>
@@ -4263,7 +4263,7 @@
         <v>160</v>
       </c>
       <c r="D67" t="n">
-        <v/>
+        <v>160</v>
       </c>
       <c r="E67" t="n">
         <v>158</v>
@@ -4313,7 +4313,7 @@
         <v>256</v>
       </c>
       <c r="D68" t="n">
-        <v/>
+        <v>256</v>
       </c>
       <c r="E68" t="n">
         <v>252</v>
@@ -4363,7 +4363,7 @@
         <v>14475</v>
       </c>
       <c r="D69" t="n">
-        <v/>
+        <v>14475</v>
       </c>
       <c r="E69" t="n">
         <v>14150</v>
@@ -4413,7 +4413,7 @@
         <v>57</v>
       </c>
       <c r="D70" t="n">
-        <v/>
+        <v>57</v>
       </c>
       <c r="E70" t="n">
         <v>53</v>
@@ -4463,7 +4463,7 @@
         <v>106</v>
       </c>
       <c r="D71" t="n">
-        <v/>
+        <v>104</v>
       </c>
       <c r="E71" t="n">
         <v>96</v>
@@ -4513,7 +4513,7 @@
         <v>64</v>
       </c>
       <c r="D72" t="n">
-        <v/>
+        <v>65</v>
       </c>
       <c r="E72" t="n">
         <v>62</v>
@@ -4563,7 +4563,7 @@
         <v>179</v>
       </c>
       <c r="D73" t="n">
-        <v/>
+        <v>174.18</v>
       </c>
       <c r="E73" t="n">
         <v>173</v>
@@ -4613,7 +4613,7 @@
         <v>143</v>
       </c>
       <c r="D74" t="n">
-        <v/>
+        <v>139.45</v>
       </c>
       <c r="E74" t="n">
         <v>126</v>
@@ -4663,7 +4663,7 @@
         <v>170</v>
       </c>
       <c r="D75" t="n">
-        <v/>
+        <v>171</v>
       </c>
       <c r="E75" t="n">
         <v>166</v>
@@ -4713,7 +4713,7 @@
         <v>294</v>
       </c>
       <c r="D76" t="n">
-        <v/>
+        <v>283.36</v>
       </c>
       <c r="E76" t="n">
         <v>286</v>
@@ -4763,7 +4763,7 @@
         <v>1250</v>
       </c>
       <c r="D77" t="n">
-        <v/>
+        <v>1250</v>
       </c>
       <c r="E77" t="n">
         <v>1250</v>
@@ -4813,7 +4813,7 @@
         <v>394</v>
       </c>
       <c r="D78" t="n">
-        <v/>
+        <v>394</v>
       </c>
       <c r="E78" t="n">
         <v>384</v>
@@ -4863,7 +4863,7 @@
         <v>166</v>
       </c>
       <c r="D79" t="n">
-        <v/>
+        <v>153.52</v>
       </c>
       <c r="E79" t="n">
         <v>153</v>
@@ -4913,7 +4913,7 @@
         <v>150</v>
       </c>
       <c r="D80" t="n">
-        <v/>
+        <v>152</v>
       </c>
       <c r="E80" t="n">
         <v>139</v>
@@ -4963,7 +4963,7 @@
         <v>1870</v>
       </c>
       <c r="D81" t="n">
-        <v/>
+        <v>1800</v>
       </c>
       <c r="E81" t="n">
         <v>1930</v>
@@ -5013,7 +5013,7 @@
         <v>488</v>
       </c>
       <c r="D82" t="n">
-        <v/>
+        <v>494</v>
       </c>
       <c r="E82" t="n">
         <v>490</v>
@@ -5063,7 +5063,7 @@
         <v>625</v>
       </c>
       <c r="D83" t="n">
-        <v/>
+        <v>630</v>
       </c>
       <c r="E83" t="n">
         <v>615</v>
@@ -5113,7 +5113,7 @@
         <v>1665</v>
       </c>
       <c r="D84" t="n">
-        <v/>
+        <v>1665</v>
       </c>
       <c r="E84" t="n">
         <v>1670</v>
@@ -5163,7 +5163,7 @@
         <v>8725</v>
       </c>
       <c r="D85" t="n">
-        <v/>
+        <v>8700</v>
       </c>
       <c r="E85" t="n">
         <v>8775</v>
@@ -5213,7 +5213,7 @@
         <v>98</v>
       </c>
       <c r="D86" t="n">
-        <v/>
+        <v>97</v>
       </c>
       <c r="E86" t="n">
         <v>93</v>
@@ -5263,7 +5263,7 @@
         <v>650</v>
       </c>
       <c r="D87" t="n">
-        <v/>
+        <v>650</v>
       </c>
       <c r="E87" t="n">
         <v>585</v>
@@ -5313,7 +5313,7 @@
         <v>178</v>
       </c>
       <c r="D88" t="n">
-        <v/>
+        <v>178</v>
       </c>
       <c r="E88" t="n">
         <v>175</v>
@@ -5363,7 +5363,7 @@
         <v>316</v>
       </c>
       <c r="D89" t="n">
-        <v/>
+        <v>316</v>
       </c>
       <c r="E89" t="n">
         <v>346</v>
@@ -5413,7 +5413,7 @@
         <v>458</v>
       </c>
       <c r="D90" t="n">
-        <v/>
+        <v>454</v>
       </c>
       <c r="E90" t="n">
         <v>448</v>
@@ -5463,7 +5463,7 @@
         <v>73</v>
       </c>
       <c r="D91" t="n">
-        <v/>
+        <v>73</v>
       </c>
       <c r="E91" t="n">
         <v>70</v>
@@ -5513,7 +5513,7 @@
         <v>1005</v>
       </c>
       <c r="D92" t="n">
-        <v/>
+        <v>1010</v>
       </c>
       <c r="E92" t="n">
         <v>1015</v>
@@ -5563,7 +5563,7 @@
         <v>2010</v>
       </c>
       <c r="D93" t="n">
-        <v/>
+        <v>2003.42</v>
       </c>
       <c r="E93" t="n">
         <v>1995</v>
@@ -5613,7 +5613,7 @@
         <v>1830</v>
       </c>
       <c r="D94" t="n">
-        <v/>
+        <v>1950</v>
       </c>
       <c r="E94" t="n">
         <v>1700</v>
@@ -5663,7 +5663,7 @@
         <v>174</v>
       </c>
       <c r="D95" t="n">
-        <v/>
+        <v>170.15</v>
       </c>
       <c r="E95" t="n">
         <v>165</v>
@@ -5713,7 +5713,7 @@
         <v>119</v>
       </c>
       <c r="D96" t="n">
-        <v/>
+        <v>118</v>
       </c>
       <c r="E96" t="n">
         <v>117</v>
@@ -5763,7 +5763,7 @@
         <v>102</v>
       </c>
       <c r="D97" t="n">
-        <v/>
+        <v>104</v>
       </c>
       <c r="E97" t="n">
         <v>101</v>
@@ -5813,7 +5813,7 @@
         <v>515</v>
       </c>
       <c r="D98" t="n">
-        <v/>
+        <v>520.7</v>
       </c>
       <c r="E98" t="n">
         <v>530</v>
@@ -5863,7 +5863,7 @@
         <v>284</v>
       </c>
       <c r="D99" t="n">
-        <v/>
+        <v>290</v>
       </c>
       <c r="E99" t="n">
         <v>268</v>
@@ -5913,7 +5913,7 @@
         <v>650</v>
       </c>
       <c r="D100" t="n">
-        <v/>
+        <v>650</v>
       </c>
       <c r="E100" t="n">
         <v>645</v>
@@ -5963,7 +5963,7 @@
         <v>112</v>
       </c>
       <c r="D101" t="n">
-        <v/>
+        <v>112</v>
       </c>
       <c r="E101" t="n">
         <v>117</v>
@@ -6013,7 +6013,7 @@
         <v>116</v>
       </c>
       <c r="D102" t="n">
-        <v/>
+        <v>127</v>
       </c>
       <c r="E102" t="n">
         <v>108</v>
@@ -6063,7 +6063,7 @@
         <v>76</v>
       </c>
       <c r="D103" t="n">
-        <v/>
+        <v>75</v>
       </c>
       <c r="E103" t="n">
         <v>70</v>
@@ -6113,7 +6113,7 @@
         <v>1550</v>
       </c>
       <c r="D104" t="n">
-        <v/>
+        <v>1550</v>
       </c>
       <c r="E104" t="n">
         <v>1705</v>
@@ -6163,7 +6163,7 @@
         <v>186</v>
       </c>
       <c r="D105" t="n">
-        <v/>
+        <v>175</v>
       </c>
       <c r="E105" t="n">
         <v>167</v>
@@ -6213,7 +6213,7 @@
         <v>58</v>
       </c>
       <c r="D106" t="n">
-        <v/>
+        <v>59</v>
       </c>
       <c r="E106" t="n">
         <v>58</v>
@@ -6263,7 +6263,7 @@
         <v>240</v>
       </c>
       <c r="D107" t="n">
-        <v/>
+        <v>236</v>
       </c>
       <c r="E107" t="n">
         <v>236</v>
@@ -6313,7 +6313,7 @@
         <v>1935</v>
       </c>
       <c r="D108" t="n">
-        <v/>
+        <v>1955</v>
       </c>
       <c r="E108" t="n">
         <v>2150</v>
@@ -6363,7 +6363,7 @@
         <v>92</v>
       </c>
       <c r="D109" t="n">
-        <v/>
+        <v>89.89</v>
       </c>
       <c r="E109" t="n">
         <v>91</v>
@@ -6413,7 +6413,7 @@
         <v>88</v>
       </c>
       <c r="D110" t="n">
-        <v/>
+        <v>88</v>
       </c>
       <c r="E110" t="n">
         <v>84</v>
@@ -6463,7 +6463,7 @@
         <v>107</v>
       </c>
       <c r="D111" t="n">
-        <v/>
+        <v>104.92</v>
       </c>
       <c r="E111" t="n">
         <v>110</v>
@@ -6513,7 +6513,7 @@
         <v>170</v>
       </c>
       <c r="D112" t="n">
-        <v/>
+        <v>173</v>
       </c>
       <c r="E112" t="n">
         <v>174</v>
@@ -6563,7 +6563,7 @@
         <v>138</v>
       </c>
       <c r="D113" t="n">
-        <v/>
+        <v>134.04</v>
       </c>
       <c r="E113" t="n">
         <v>137</v>
@@ -6613,7 +6613,7 @@
         <v>570</v>
       </c>
       <c r="D114" t="n">
-        <v/>
+        <v>570</v>
       </c>
       <c r="E114" t="n">
         <v>570</v>
@@ -6663,7 +6663,7 @@
         <v>140</v>
       </c>
       <c r="D115" t="n">
-        <v/>
+        <v>142</v>
       </c>
       <c r="E115" t="n">
         <v>139</v>
@@ -6713,7 +6713,7 @@
         <v>108</v>
       </c>
       <c r="D116" t="n">
-        <v/>
+        <v>108</v>
       </c>
       <c r="E116" t="n">
         <v>123</v>
@@ -6763,7 +6763,7 @@
         <v>875</v>
       </c>
       <c r="D117" t="n">
-        <v/>
+        <v>871.55</v>
       </c>
       <c r="E117" t="n">
         <v>845</v>
@@ -6813,7 +6813,7 @@
         <v>376</v>
       </c>
       <c r="D118" t="n">
-        <v/>
+        <v>376</v>
       </c>
       <c r="E118" t="n">
         <v>372</v>
@@ -6863,7 +6863,7 @@
         <v>89</v>
       </c>
       <c r="D119" t="n">
-        <v/>
+        <v>89</v>
       </c>
       <c r="E119" t="n">
         <v>89</v>
@@ -6913,7 +6913,7 @@
         <v>875</v>
       </c>
       <c r="D120" t="n">
-        <v/>
+        <v>865</v>
       </c>
       <c r="E120" t="n">
         <v>870</v>
@@ -6963,7 +6963,7 @@
         <v>855</v>
       </c>
       <c r="D121" t="n">
-        <v/>
+        <v>830</v>
       </c>
       <c r="E121" t="n">
         <v>810</v>
@@ -7013,7 +7013,7 @@
         <v>130</v>
       </c>
       <c r="D122" t="n">
-        <v/>
+        <v>135</v>
       </c>
       <c r="E122" t="n">
         <v>141</v>
@@ -7063,7 +7063,7 @@
         <v>183</v>
       </c>
       <c r="D123" t="n">
-        <v/>
+        <v>184</v>
       </c>
       <c r="E123" t="n">
         <v>180</v>
@@ -7113,7 +7113,7 @@
         <v>89</v>
       </c>
       <c r="D124" t="n">
-        <v/>
+        <v>89</v>
       </c>
       <c r="E124" t="n">
         <v>86</v>
@@ -7163,7 +7163,7 @@
         <v>1480</v>
       </c>
       <c r="D125" t="n">
-        <v/>
+        <v>1480</v>
       </c>
       <c r="E125" t="n">
         <v>1450</v>
@@ -7213,7 +7213,7 @@
         <v>208</v>
       </c>
       <c r="D126" t="n">
-        <v/>
+        <v>208</v>
       </c>
       <c r="E126" t="n">
         <v>206</v>
@@ -7263,7 +7263,7 @@
         <v>116</v>
       </c>
       <c r="D127" t="n">
-        <v/>
+        <v>115</v>
       </c>
       <c r="E127" t="n">
         <v>117</v>
@@ -7313,7 +7313,7 @@
         <v>965</v>
       </c>
       <c r="D128" t="n">
-        <v/>
+        <v>915.12</v>
       </c>
       <c r="E128" t="n">
         <v>910</v>
@@ -7363,7 +7363,7 @@
         <v>515</v>
       </c>
       <c r="D129" t="n">
-        <v/>
+        <v>515</v>
       </c>
       <c r="E129" t="n">
         <v>535</v>
@@ -7413,7 +7413,7 @@
         <v>282</v>
       </c>
       <c r="D130" t="n">
-        <v/>
+        <v>274</v>
       </c>
       <c r="E130" t="n">
         <v>268</v>
@@ -7463,7 +7463,7 @@
         <v>246</v>
       </c>
       <c r="D131" t="n">
-        <v/>
+        <v>256</v>
       </c>
       <c r="E131" t="n">
         <v>238</v>
@@ -7513,7 +7513,7 @@
         <v>91</v>
       </c>
       <c r="D132" t="n">
-        <v/>
+        <v>92</v>
       </c>
       <c r="E132" t="n">
         <v>90</v>

</xml_diff>